<commit_message>
added changes to lang and english template
</commit_message>
<xml_diff>
--- a/src/R/Modals/configrm_lang.xlsx
+++ b/src/R/Modals/configrm_lang.xlsx
@@ -374,7 +374,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>QA correcto</t>
+          <t>QA correct</t>
         </is>
       </c>
     </row>
@@ -386,7 +386,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>QA incorrecto</t>
+          <t>QA incorrect</t>
         </is>
       </c>
     </row>
@@ -398,7 +398,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>QA Reporte</t>
+          <t>QA report</t>
         </is>
       </c>
     </row>
@@ -410,7 +410,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Descargar reporte</t>
+          <t>Download report</t>
         </is>
       </c>
     </row>
@@ -422,7 +422,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>El reporte de QA no ha encontrado errores en los datos.</t>
+          <t>QA report found no errors in the data.</t>
         </is>
       </c>
     </row>
@@ -434,7 +434,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>El reporte de QA ha encontrado errores en los datos, revisar detalles en el informe de reporte.</t>
+          <t>QA report found errors in the data. Check details in the report.</t>
         </is>
       </c>
     </row>
@@ -446,7 +446,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Configuración correcta</t>
+          <t>Correct configuration</t>
         </is>
       </c>
     </row>
@@ -458,7 +458,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Configuración incorrecta</t>
+          <t>Incorrect configuration</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Todos los paquetes fueron instalados</t>
+          <t>All packets were installed</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Algunos paquetes no fueron instalados:</t>
+          <t>Some packets were not installed:</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cerrar</t>
+          <t>Close</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added mediation and downloadable report logic
</commit_message>
<xml_diff>
--- a/src/R/Modals/configrm_lang.xlsx
+++ b/src/R/Modals/configrm_lang.xlsx
@@ -374,7 +374,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>QA correct</t>
+          <t>QA correcto</t>
         </is>
       </c>
     </row>
@@ -386,7 +386,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>QA incorrect</t>
+          <t>QA incorrecto</t>
         </is>
       </c>
     </row>
@@ -398,7 +398,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>QA report</t>
+          <t>QA Reporte</t>
         </is>
       </c>
     </row>
@@ -410,7 +410,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Download report</t>
+          <t>Descargar reporte</t>
         </is>
       </c>
     </row>
@@ -422,7 +422,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>QA report found no errors in the data.</t>
+          <t>El reporte de QA no ha encontrado errores en los datos.</t>
         </is>
       </c>
     </row>
@@ -434,7 +434,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>QA report found errors in the data. Check details in the report.</t>
+          <t>El reporte de QA ha encontrado errores en los datos, revisar detalles en el informe de reporte.</t>
         </is>
       </c>
     </row>
@@ -446,7 +446,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Correct configuration</t>
+          <t>Configuración correcta</t>
         </is>
       </c>
     </row>
@@ -458,7 +458,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Incorrect configuration</t>
+          <t>Configuración incorrecta</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>All packets were installed</t>
+          <t>Todos los paquetes fueron instalados</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Some packets were not installed:</t>
+          <t>Algunos paquetes no fueron instalados:</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Cerrar</t>
         </is>
       </c>
     </row>

</xml_diff>